<commit_message>
fix(pro-novinare): vypořádání review Codexu u 2. kola, kolo 1
- Stránka neodvozuje z podobných počtů, kolik dětí z 1. kola zkusilo
  2. kolo; překryv výslovně nelze určit.
- Sloupec z_toho_jiny_duvod, rozklad důvodů sedí na součet (+test).
- Slovník bez zástupného {rok}.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/pro-novinare/uchazeci-2026.xlsx
+++ b/public/pro-novinare/uchazeci-2026.xlsx
@@ -2682,7 +2682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2694,11 +2694,12 @@
     <col width="37" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="38" customWidth="1" min="13" max="13"/>
-    <col width="29" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="29" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2749,25 +2750,30 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
+          <t>z_toho_jiny_duvod</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
           <t>z_toho_hlasili_se_jen_na_obory_bez_maturity</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>z_toho_jen_na_maturitni</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>z_toho_na_oboje</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>z_toho_bez_vysledku_jednotne_zkousky</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>z_toho_s_jedinou_prihlaskou</t>
         </is>
@@ -2806,18 +2812,21 @@
         <v>336</v>
       </c>
       <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
         <v>366</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>279</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>140</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>368</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>75</v>
       </c>
     </row>
@@ -2857,15 +2866,18 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
         <v>129</v>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
       <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>79</v>
       </c>
     </row>
@@ -2905,15 +2917,18 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
         <v>117</v>
       </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
       <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>79</v>
       </c>
     </row>
@@ -2950,18 +2965,21 @@
         <v>22</v>
       </c>
       <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
         <v>46</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>55</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>10</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>65</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>35</v>
       </c>
     </row>
@@ -3001,15 +3019,18 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
         <v>26</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
       <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
         <v>3</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3046,18 +3067,21 @@
         <v>2</v>
       </c>
       <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
         <v>12</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>4</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>2</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>10</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3097,15 +3121,18 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
         <v>5</v>
       </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3142,18 +3169,21 @@
         <v>11</v>
       </c>
       <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
         <v>45</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>10</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>6</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>45</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3190,18 +3220,21 @@
         <v>3</v>
       </c>
       <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
         <v>7</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>3</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>2</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>7</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3241,15 +3274,18 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
         <v>4</v>
       </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3286,18 +3322,21 @@
         <v>11</v>
       </c>
       <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
         <v>42</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>18</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>5</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>50</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3337,15 +3376,18 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
         <v>15</v>
       </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
         <v>13</v>
       </c>
     </row>
@@ -3382,18 +3424,21 @@
         <v>37</v>
       </c>
       <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
         <v>106</v>
-      </c>
-      <c r="K14" t="n">
-        <v>15</v>
       </c>
       <c r="L14" t="n">
         <v>15</v>
       </c>
       <c r="M14" t="n">
+        <v>15</v>
+      </c>
+      <c r="N14" t="n">
         <v>106</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>53</v>
       </c>
     </row>
@@ -3433,15 +3478,18 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
         <v>9</v>
       </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
       <c r="M15" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3478,18 +3526,21 @@
         <v>8</v>
       </c>
       <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
         <v>30</v>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>15</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>3</v>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>41</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>28</v>
       </c>
     </row>
@@ -3529,15 +3580,18 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
         <v>33</v>
       </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
       <c r="M17" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3577,15 +3631,18 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
         <v>25</v>
       </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
       <c r="M18" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3622,18 +3679,21 @@
         <v>4</v>
       </c>
       <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
         <v>28</v>
       </c>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>11</v>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>4</v>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>38</v>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3673,15 +3733,18 @@
         <v>0</v>
       </c>
       <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
         <v>13</v>
       </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
       <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
         <v>2</v>
       </c>
-      <c r="N20" t="n">
+      <c r="O20" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3718,18 +3781,21 @@
         <v>7</v>
       </c>
       <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
         <v>21</v>
       </c>
-      <c r="K21" t="n">
+      <c r="L21" t="n">
         <v>16</v>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>5</v>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>22</v>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>17</v>
       </c>
     </row>
@@ -3769,15 +3835,18 @@
         <v>0</v>
       </c>
       <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
         <v>26</v>
       </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
       <c r="M22" t="n">
         <v>0</v>
       </c>
       <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
         <v>21</v>
       </c>
     </row>
@@ -3814,18 +3883,21 @@
         <v>22</v>
       </c>
       <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="n">
         <v>29</v>
       </c>
-      <c r="K23" t="n">
+      <c r="L23" t="n">
         <v>23</v>
       </c>
-      <c r="L23" t="n">
+      <c r="M23" t="n">
         <v>11</v>
       </c>
-      <c r="M23" t="n">
+      <c r="N23" t="n">
         <v>39</v>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3865,15 +3937,18 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
         <v>7</v>
       </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
       <c r="M24" t="n">
         <v>0</v>
       </c>
       <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
         <v>7</v>
       </c>
     </row>
@@ -3910,18 +3985,21 @@
         <v>93</v>
       </c>
       <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
         <v>164</v>
       </c>
-      <c r="K25" t="n">
+      <c r="L25" t="n">
         <v>73</v>
       </c>
-      <c r="L25" t="n">
+      <c r="M25" t="n">
         <v>43</v>
       </c>
-      <c r="M25" t="n">
+      <c r="N25" t="n">
         <v>163</v>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>52</v>
       </c>
     </row>
@@ -3961,15 +4039,18 @@
         <v>0</v>
       </c>
       <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
         <v>29</v>
       </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
       <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
         <v>1</v>
       </c>
-      <c r="N26" t="n">
+      <c r="O26" t="n">
         <v>29</v>
       </c>
     </row>
@@ -4006,18 +4087,21 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
         <v>11</v>
       </c>
-      <c r="K27" t="n">
+      <c r="L27" t="n">
         <v>3</v>
       </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
       <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
         <v>11</v>
       </c>
-      <c r="N27" t="n">
+      <c r="O27" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4057,15 +4141,18 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
         <v>12</v>
       </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
       <c r="M28" t="n">
         <v>0</v>
       </c>
       <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4105,15 +4192,18 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
         <v>5</v>
       </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
       <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
         <v>1</v>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4150,18 +4240,21 @@
         <v>17</v>
       </c>
       <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
         <v>69</v>
       </c>
-      <c r="K30" t="n">
+      <c r="L30" t="n">
         <v>20</v>
       </c>
-      <c r="L30" t="n">
+      <c r="M30" t="n">
         <v>4</v>
       </c>
-      <c r="M30" t="n">
+      <c r="N30" t="n">
         <v>81</v>
       </c>
-      <c r="N30" t="n">
+      <c r="O30" t="n">
         <v>42</v>
       </c>
     </row>
@@ -4201,15 +4294,18 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
         <v>13</v>
       </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
       <c r="M31" t="n">
         <v>0</v>
       </c>
       <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4249,15 +4345,18 @@
         <v>0</v>
       </c>
       <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
         <v>8</v>
       </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
       <c r="M32" t="n">
         <v>0</v>
       </c>
       <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4272,7 +4371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4284,11 +4383,12 @@
     <col width="37" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="38" customWidth="1" min="13" max="13"/>
-    <col width="29" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
+    <col width="29" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4339,25 +4439,30 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
+          <t>z_toho_jiny_duvod</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
           <t>z_toho_hlasili_se_jen_na_obory_bez_maturity</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>z_toho_jen_na_maturitni</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>z_toho_na_oboje</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>z_toho_bez_vysledku_jednotne_zkousky</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>z_toho_s_jedinou_prihlaskou</t>
         </is>
@@ -4396,18 +4501,21 @@
         <v>573</v>
       </c>
       <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
         <v>976</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>545</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>250</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>1046</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>407</v>
       </c>
     </row>
@@ -4447,15 +4555,18 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
         <v>191</v>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
       <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
         <v>1</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>123</v>
       </c>
     </row>
@@ -4495,15 +4606,18 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
         <v>285</v>
       </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
       <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
         <v>12</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>216</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(pro-novinare): vypořádání review Codexu u 2. kola, kolo 3
Kraj uchazeče podle školy a oboru, ne jen podle REDIZO (PORG má obory
v Jihomoravském i Moravskoslezském kraji); nejednoznačná dvojice jde
do řádku „kraj neurčen“. Platí pro 1. i 2. kolo; test.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/pro-novinare/uchazeci-2026.xlsx
+++ b/public/pro-novinare/uchazeci-2026.xlsx
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -652,34 +652,34 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>19910</v>
+        <v>19975</v>
       </c>
       <c r="D2" t="n">
-        <v>16178</v>
+        <v>16240</v>
       </c>
       <c r="E2" t="n">
-        <v>10512</v>
+        <v>10536</v>
       </c>
       <c r="F2" t="n">
-        <v>3661</v>
+        <v>3691</v>
       </c>
       <c r="G2" t="n">
-        <v>2371</v>
+        <v>2377</v>
       </c>
       <c r="H2" t="n">
-        <v>3366</v>
+        <v>3371</v>
       </c>
       <c r="I2" t="n">
         <v>0.169</v>
       </c>
       <c r="J2" t="n">
-        <v>964</v>
+        <v>967</v>
       </c>
       <c r="K2" t="n">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="L2" t="n">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -787,34 +787,34 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12549</v>
+        <v>12484</v>
       </c>
       <c r="D5" t="n">
-        <v>9319</v>
+        <v>9257</v>
       </c>
       <c r="E5" t="n">
-        <v>8258</v>
+        <v>8234</v>
       </c>
       <c r="F5" t="n">
-        <v>2099</v>
+        <v>2069</v>
       </c>
       <c r="G5" t="n">
-        <v>1155</v>
+        <v>1149</v>
       </c>
       <c r="H5" t="n">
-        <v>1037</v>
+        <v>1032</v>
       </c>
       <c r="I5" t="n">
         <v>0.083</v>
       </c>
       <c r="J5" t="n">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="K5" t="n">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L5" t="n">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -877,34 +877,34 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2709</v>
+        <v>2452</v>
       </c>
       <c r="D7" t="n">
-        <v>2623</v>
+        <v>2370</v>
       </c>
       <c r="E7" t="n">
-        <v>880</v>
+        <v>763</v>
       </c>
       <c r="F7" t="n">
-        <v>175</v>
+        <v>143</v>
       </c>
       <c r="G7" t="n">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="H7" t="n">
-        <v>1570</v>
+        <v>1483</v>
       </c>
       <c r="I7" t="n">
-        <v>0.58</v>
+        <v>0.605</v>
       </c>
       <c r="J7" t="n">
-        <v>801</v>
+        <v>757</v>
       </c>
       <c r="K7" t="n">
-        <v>274</v>
+        <v>256</v>
       </c>
       <c r="L7" t="n">
-        <v>495</v>
+        <v>470</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -2308,43 +2308,43 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ústecký kraj</t>
+          <t>kraj neurčen (škola má obor ve více krajích)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>9. třída (čtyřleté obory a obory bez maturity)</t>
+          <t>5. třída (osmiletá gymnázia)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>8800</v>
+        <v>257</v>
       </c>
       <c r="D39" t="n">
-        <v>5700</v>
+        <v>253</v>
       </c>
       <c r="E39" t="n">
-        <v>6997</v>
+        <v>117</v>
       </c>
       <c r="F39" t="n">
-        <v>989</v>
+        <v>32</v>
       </c>
       <c r="G39" t="n">
-        <v>397</v>
+        <v>21</v>
       </c>
       <c r="H39" t="n">
-        <v>417</v>
+        <v>87</v>
       </c>
       <c r="I39" t="n">
-        <v>0.047</v>
+        <v>0.339</v>
       </c>
       <c r="J39" t="n">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="K39" t="n">
-        <v>156</v>
+        <v>18</v>
       </c>
       <c r="L39" t="n">
-        <v>165</v>
+        <v>25</v>
       </c>
       <c r="M39" t="n">
         <v>0</v>
@@ -2358,38 +2358,38 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>7. třída (šestiletá gymnázia)</t>
+          <t>9. třída (čtyřleté obory a obory bez maturity)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>63</v>
+        <v>8800</v>
       </c>
       <c r="D40" t="n">
-        <v>63</v>
+        <v>5700</v>
       </c>
       <c r="E40" t="n">
-        <v>30</v>
+        <v>6997</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>989</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>397</v>
       </c>
       <c r="H40" t="n">
-        <v>33</v>
+        <v>417</v>
       </c>
       <c r="I40" t="n">
-        <v>0.524</v>
+        <v>0.047</v>
       </c>
       <c r="J40" t="n">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="K40" t="n">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="M40" t="n">
         <v>0</v>
@@ -2403,40 +2403,85 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>7. třída (šestiletá gymnázia)</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>63</v>
+      </c>
+      <c r="D41" t="n">
+        <v>63</v>
+      </c>
+      <c r="E41" t="n">
+        <v>30</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>33</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="J41" t="n">
+        <v>12</v>
+      </c>
+      <c r="K41" t="n">
+        <v>21</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ústecký kraj</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>5. třída (osmiletá gymnázia)</t>
         </is>
       </c>
-      <c r="C41" t="n">
+      <c r="C42" t="n">
         <v>916</v>
       </c>
-      <c r="D41" t="n">
+      <c r="D42" t="n">
         <v>883</v>
       </c>
-      <c r="E41" t="n">
+      <c r="E42" t="n">
         <v>518</v>
       </c>
-      <c r="F41" t="n">
+      <c r="F42" t="n">
         <v>41</v>
       </c>
-      <c r="G41" t="n">
+      <c r="G42" t="n">
         <v>13</v>
       </c>
-      <c r="H41" t="n">
+      <c r="H42" t="n">
         <v>344</v>
       </c>
-      <c r="I41" t="n">
+      <c r="I42" t="n">
         <v>0.376</v>
       </c>
-      <c r="J41" t="n">
+      <c r="J42" t="n">
         <v>290</v>
       </c>
-      <c r="K41" t="n">
+      <c r="K42" t="n">
         <v>45</v>
       </c>
-      <c r="L41" t="n">
+      <c r="L42" t="n">
         <v>9</v>
       </c>
-      <c r="M41" t="n">
+      <c r="M42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2944,10 +2989,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1154</v>
+        <v>1158</v>
       </c>
       <c r="D5" t="n">
-        <v>1043</v>
+        <v>1047</v>
       </c>
       <c r="E5" t="n">
         <v>111</v>
@@ -3505,10 +3550,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>877</v>
+        <v>873</v>
       </c>
       <c r="D16" t="n">
-        <v>829</v>
+        <v>825</v>
       </c>
       <c r="E16" t="n">
         <v>48</v>

</xml_diff>